<commit_message>
Yan branch (#12) update plot result
* add plot result

* add plot result

* update get_data_stats.py

* plot_result.py add error bar

* add plot result

* update get_data_stats.py

* plot_result.py add error bar
</commit_message>
<xml_diff>
--- a/src/process_exp_result/processed_result/processed/DNABert2_results.xlsx
+++ b/src/process_exp_result/processed_result/processed/DNABert2_results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yanzhang\Desktop\GeneLLM\src\process_exp_result\processed_result\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yanzhang\Desktop\GeneLLM\src\process_exp_result\processed_result\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76AF37A-C94A-4F6D-A832-400A3C4EF103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25938D9-2693-4C92-AD77-6F3D037B06D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="1950" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,12 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="36">
   <si>
-    <t>task_name</t>
-  </si>
-  <si>
-    <t>subset_name</t>
-  </si>
-  <si>
     <t>EMP</t>
   </si>
   <si>
@@ -135,6 +129,14 @@
   </si>
   <si>
     <t>test_F1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>task_name_test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>subset_name_test</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -499,31 +501,31 @@
   <dimension ref="A1:D29"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.58203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>57.42</v>
@@ -531,10 +533,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C3">
         <v>61.9</v>
@@ -542,10 +544,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
       </c>
       <c r="C4">
         <v>53</v>
@@ -553,10 +555,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C5">
         <v>39.89</v>
@@ -564,10 +566,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C6">
         <v>41.2</v>
@@ -575,10 +577,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C7">
         <v>65.64</v>
@@ -586,10 +588,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C8">
         <v>57.07</v>
@@ -597,10 +599,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C9">
         <v>80.17</v>
@@ -608,10 +610,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C10">
         <v>50.35</v>
@@ -619,10 +621,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C11">
         <v>81.86</v>
@@ -630,10 +632,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C12">
         <v>64.23</v>
@@ -641,10 +643,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
         <v>14</v>
-      </c>
-      <c r="B13" t="s">
-        <v>16</v>
       </c>
       <c r="C13">
         <v>86.28</v>
@@ -652,10 +654,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C14">
         <v>81.28</v>
@@ -663,10 +665,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C15">
         <v>73.489999999999995</v>
@@ -674,10 +676,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C16">
         <v>50.8</v>
@@ -685,10 +687,10 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C17">
         <v>88.31</v>
@@ -696,10 +698,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
         <v>20</v>
-      </c>
-      <c r="B18" t="s">
-        <v>22</v>
       </c>
       <c r="C18">
         <v>94.34</v>
@@ -707,10 +709,10 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C19">
         <v>68.790000000000006</v>
@@ -718,10 +720,10 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C20">
         <v>67.5</v>
@@ -729,10 +731,10 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C21">
         <v>69.53</v>
@@ -740,10 +742,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B22" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C22">
         <v>76.180000000000007</v>
@@ -751,10 +753,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C23">
         <v>85.93</v>
@@ -762,10 +764,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C24">
         <v>69.12</v>
@@ -773,10 +775,10 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" t="s">
         <v>27</v>
-      </c>
-      <c r="B25" t="s">
-        <v>29</v>
       </c>
       <c r="C25">
         <v>71.87</v>
@@ -784,10 +786,10 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C26">
         <v>62.96</v>
@@ -795,10 +797,10 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C27">
         <v>55.35</v>
@@ -806,10 +808,10 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C28">
         <v>74.94</v>
@@ -817,10 +819,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D29">
         <v>68.489999999999995</v>

</xml_diff>